<commit_message>
Corrigir Mega Sena - adicionar concurso 3031 (14/07/2026) que estava faltando
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/timemania_asloterias_ate_concurso_2414_crescente.xlsx
+++ b/historicoresultadosloteriasnacionais/timemania_asloterias_ate_concurso_2414_crescente.xlsx
@@ -413,37 +413,99 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
+        <v>2416</v>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C1" t="n">
+        <v>17</v>
+      </c>
+      <c r="D1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1" t="n">
+        <v>36</v>
+      </c>
+      <c r="F1" t="n">
+        <v>50</v>
+      </c>
+      <c r="G1" t="n">
+        <v>70</v>
+      </c>
+      <c r="H1" t="n">
+        <v>74</v>
+      </c>
+      <c r="I1" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2415</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>11</v>
+      </c>
+      <c r="F2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H2" t="n">
+        <v>44</v>
+      </c>
+      <c r="I2" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>2414</v>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="C1" t="n">
+      <c r="C3" t="n">
         <v>18</v>
       </c>
-      <c r="D1" t="n">
+      <c r="D3" t="n">
         <v>19</v>
       </c>
-      <c r="E1" t="n">
+      <c r="E3" t="n">
         <v>36</v>
       </c>
-      <c r="F1" t="n">
+      <c r="F3" t="n">
         <v>63</v>
       </c>
-      <c r="G1" t="n">
+      <c r="G3" t="n">
         <v>64</v>
       </c>
-      <c r="H1" t="n">
+      <c r="H3" t="n">
         <v>67</v>
       </c>
-      <c r="I1" t="n">
+      <c r="I3" t="n">
         <v>71</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adicionar concursos faltantes da Mega-Sena (3034-3040)
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/timemania_asloterias_ate_concurso_2414_crescente.xlsx
+++ b/historicoresultadosloteriasnacionais/timemania_asloterias_ate_concurso_2414_crescente.xlsx
@@ -413,99 +413,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>2416</v>
+        <v>2422</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C1" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D1" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="E1" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="F1" t="n">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="G1" t="n">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="H1" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="I1" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2415</v>
+        <v>2421</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F2" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="G2" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="H2" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="I2" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>2420</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F3" t="n">
+        <v>72</v>
+      </c>
+      <c r="G3" t="n">
+        <v>76</v>
+      </c>
+      <c r="H3" t="n">
+        <v>77</v>
+      </c>
+      <c r="I3" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2419</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>26</v>
+      </c>
+      <c r="G4" t="n">
+        <v>48</v>
+      </c>
+      <c r="H4" t="n">
+        <v>52</v>
+      </c>
+      <c r="I4" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2418</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E5" t="n">
+        <v>45</v>
+      </c>
+      <c r="F5" t="n">
+        <v>67</v>
+      </c>
+      <c r="G5" t="n">
+        <v>71</v>
+      </c>
+      <c r="H5" t="n">
+        <v>74</v>
+      </c>
+      <c r="I5" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2416</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" t="n">
+        <v>36</v>
+      </c>
+      <c r="F6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G6" t="n">
+        <v>70</v>
+      </c>
+      <c r="H6" t="n">
+        <v>74</v>
+      </c>
+      <c r="I6" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2415</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F7" t="n">
+        <v>21</v>
+      </c>
+      <c r="G7" t="n">
+        <v>42</v>
+      </c>
+      <c r="H7" t="n">
+        <v>44</v>
+      </c>
+      <c r="I7" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
         <v>2414</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C8" t="n">
         <v>18</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D8" t="n">
         <v>19</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E8" t="n">
         <v>36</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F8" t="n">
         <v>63</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G8" t="n">
         <v>64</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H8" t="n">
         <v>67</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I8" t="n">
         <v>71</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizar todas as loterias com concursos faltantes
</commit_message>
<xml_diff>
--- a/historicoresultadosloteriasnacionais/timemania_asloterias_ate_concurso_2414_crescente.xlsx
+++ b/historicoresultadosloteriasnacionais/timemania_asloterias_ate_concurso_2414_crescente.xlsx
@@ -413,254 +413,378 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>2422</v>
+        <v>2417</v>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="C1" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D1" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E1" t="n">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" t="n">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="G1" t="n">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="H1" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="I1" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2421</v>
+        <v>2425</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="F2" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="G2" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="H2" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="I2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2420</v>
+        <v>2424</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F3" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="G3" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="H3" t="n">
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="I3" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2419</v>
+        <v>2423</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G4" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H4" t="n">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="I4" t="n">
-        <v>59</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2418</v>
+        <v>2422</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
         <v>19</v>
       </c>
       <c r="E5" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="F5" t="n">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="G5" t="n">
-        <v>71</v>
+        <v>34</v>
       </c>
       <c r="H5" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="I5" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2416</v>
+        <v>2421</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E6" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F6" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G6" t="n">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="H6" t="n">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="I6" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2415</v>
+        <v>2420</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F7" t="n">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="G7" t="n">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="H7" t="n">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="I7" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>2419</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>26</v>
+      </c>
+      <c r="G8" t="n">
+        <v>48</v>
+      </c>
+      <c r="H8" t="n">
+        <v>52</v>
+      </c>
+      <c r="I8" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2418</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G9" t="n">
+        <v>71</v>
+      </c>
+      <c r="H9" t="n">
+        <v>74</v>
+      </c>
+      <c r="I9" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2416</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>17</v>
+      </c>
+      <c r="D10" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" t="n">
+        <v>36</v>
+      </c>
+      <c r="F10" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" t="n">
+        <v>70</v>
+      </c>
+      <c r="H10" t="n">
+        <v>74</v>
+      </c>
+      <c r="I10" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2415</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="n">
+        <v>11</v>
+      </c>
+      <c r="F11" t="n">
+        <v>21</v>
+      </c>
+      <c r="G11" t="n">
+        <v>42</v>
+      </c>
+      <c r="H11" t="n">
+        <v>44</v>
+      </c>
+      <c r="I11" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
         <v>2414</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C12" t="n">
         <v>18</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D12" t="n">
         <v>19</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E12" t="n">
         <v>36</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F12" t="n">
         <v>63</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G12" t="n">
         <v>64</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H12" t="n">
         <v>67</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I12" t="n">
         <v>71</v>
       </c>
     </row>

</xml_diff>